<commit_message>
Add runnable NVIDIA models to the registry
nemotron-super-49b was in the registry but had a blank ollama_tag, so it never
appeared in a run - a bad gap for a DGX benchmark. The Super-49B is not in the
Ollama library, so rather than mislabel that row with a different model's tag,
add the two NVIDIA models that are:

- nemotron-70b (nemotron:70b), NVIDIA's RLHF tune of Llama 3.1 70B. Same size and
  family as llama-3.3-70b, so it is a direct A/B on identical hardware.
- nemotron-mini-4b (nemotron-mini:4b), small-model efficiency reference. Its 4k
  context means the longer ISL/OSL shapes are skipped automatically.

nemotron-super-49b keeps a blank tag and is now annotated vLLM/TRT-LLM only.
Registry is 26 models; 11 are runnable via Ollama once China is excluded.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dgx_llm_benchmark.xlsx
+++ b/dgx_llm_benchmark.xlsx
@@ -20,7 +20,7 @@
     <sheet name="Summary" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Models!$A$4:$R$27</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Models!$A$4:$R$29</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Ollama_Pull_Log!$A$4:$K$404</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Parameters!$A$4:$H$78</definedName>
     <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">Perf_Results!$A$1:$AZ$400</definedName>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="798">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="810">
   <si>
     <t xml:space="preserve">DGX LLM Benchmark - data collection workbook</t>
   </si>
@@ -1921,7 +1921,49 @@
     <t xml:space="preserve">nvidia/Llama-3_3-Nemotron-Super-49B-v1</t>
   </si>
   <si>
-    <t xml:space="preserve">NVIDIA-tuned; expect best TRT-LLM numbers</t>
+    <t xml:space="preserve">NVIDIA-tuned; expect best TRT-LLM numbers. No Ollama tag - vLLM/TRT-LLM only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nemotron-70b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Llama 3.1 Nemotron 70B Instruct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NVIDIA Open Model / Llama 3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nvidia/Llama-3.1-Nemotron-70B-Instruct-HF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nemotron:70b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NVIDIA RLHF tune of Llama 3.1 70B. Direct A/B against llama-3.3-70b on the same hardware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nemotron-mini-4b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nemotron Mini 4B Instruct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NVIDIA Community</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nvidia/Nemotron-Mini-4B-Instruct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nemotron-mini:4b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BF16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small-model efficiency reference; short context limits which shapes apply</t>
   </si>
   <si>
     <t xml:space="preserve">olmo-2-32b</t>
@@ -1934,12 +1976,6 @@
   </si>
   <si>
     <t xml:space="preserve">allenai/OLMo-2-0325-32B-Instruct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BF16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2</t>
   </si>
   <si>
     <t xml:space="preserve">Fully open data/training - reproducibility reference</t>
@@ -3452,7 +3488,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -3470,12 +3506,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>783</v>
+        <v>795</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>784</v>
+        <v>796</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3492,40 +3528,40 @@
         <v>524</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>785</v>
+        <v>797</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>786</v>
+        <v>798</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>787</v>
+        <v>799</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>788</v>
+        <v>800</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>789</v>
+        <v>801</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>790</v>
+        <v>802</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>791</v>
+        <v>803</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>792</v>
+        <v>804</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>793</v>
+        <v>805</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>794</v>
+        <v>806</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>795</v>
+        <v>807</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>796</v>
+        <v>808</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4191,15 +4227,15 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="29" t="str">
         <f aca="false">IF(Models!A15="","",Models!A15)</f>
-        <v>olmo-2-32b</v>
+        <v>nemotron-70b</v>
       </c>
       <c r="B15" s="29" t="str">
         <f aca="false">IF(Models!B15="","",Models!B15)</f>
-        <v>OLMo 2 32B Instruct</v>
+        <v>Llama 3.1 Nemotron 70B Instruct</v>
       </c>
       <c r="C15" s="29" t="str">
         <f aca="false">IF(Models!C15="","",Models!C15)</f>
-        <v>Allen Institute (AI2)</v>
+        <v>NVIDIA</v>
       </c>
       <c r="D15" s="29" t="str">
         <f aca="false">IF(Models!D15="","",Models!D15)</f>
@@ -4257,19 +4293,19 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="29" t="str">
         <f aca="false">IF(Models!A16="","",Models!A16)</f>
-        <v>mistral-small-3</v>
+        <v>nemotron-mini-4b</v>
       </c>
       <c r="B16" s="29" t="str">
         <f aca="false">IF(Models!B16="","",Models!B16)</f>
-        <v>Mistral Small 3.x Instruct</v>
+        <v>Nemotron Mini 4B Instruct</v>
       </c>
       <c r="C16" s="29" t="str">
         <f aca="false">IF(Models!C16="","",Models!C16)</f>
-        <v>Mistral AI</v>
+        <v>NVIDIA</v>
       </c>
       <c r="D16" s="29" t="str">
         <f aca="false">IF(Models!D16="","",Models!D16)</f>
-        <v>France</v>
+        <v>USA</v>
       </c>
       <c r="E16" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A16)</f>
@@ -4323,19 +4359,19 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="29" t="str">
         <f aca="false">IF(Models!A17="","",Models!A17)</f>
-        <v>mixtral-8x22b</v>
+        <v>olmo-2-32b</v>
       </c>
       <c r="B17" s="29" t="str">
         <f aca="false">IF(Models!B17="","",Models!B17)</f>
-        <v>Mixtral 8x22B Instruct</v>
+        <v>OLMo 2 32B Instruct</v>
       </c>
       <c r="C17" s="29" t="str">
         <f aca="false">IF(Models!C17="","",Models!C17)</f>
-        <v>Mistral AI</v>
+        <v>Allen Institute (AI2)</v>
       </c>
       <c r="D17" s="29" t="str">
         <f aca="false">IF(Models!D17="","",Models!D17)</f>
-        <v>France</v>
+        <v>USA</v>
       </c>
       <c r="E17" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A17)</f>
@@ -4389,19 +4425,19 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="29" t="str">
         <f aca="false">IF(Models!A18="","",Models!A18)</f>
-        <v>glm-4.5</v>
+        <v>mistral-small-3</v>
       </c>
       <c r="B18" s="29" t="str">
         <f aca="false">IF(Models!B18="","",Models!B18)</f>
-        <v>GLM-4.5</v>
+        <v>Mistral Small 3.x Instruct</v>
       </c>
       <c r="C18" s="29" t="str">
         <f aca="false">IF(Models!C18="","",Models!C18)</f>
-        <v>Zhipu AI / Z.ai</v>
+        <v>Mistral AI</v>
       </c>
       <c r="D18" s="29" t="str">
         <f aca="false">IF(Models!D18="","",Models!D18)</f>
-        <v>China</v>
+        <v>France</v>
       </c>
       <c r="E18" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A18)</f>
@@ -4455,19 +4491,19 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="29" t="str">
         <f aca="false">IF(Models!A19="","",Models!A19)</f>
-        <v>kimi-k2</v>
+        <v>mixtral-8x22b</v>
       </c>
       <c r="B19" s="29" t="str">
         <f aca="false">IF(Models!B19="","",Models!B19)</f>
-        <v>Kimi K2 Instruct</v>
+        <v>Mixtral 8x22B Instruct</v>
       </c>
       <c r="C19" s="29" t="str">
         <f aca="false">IF(Models!C19="","",Models!C19)</f>
-        <v>Moonshot AI</v>
+        <v>Mistral AI</v>
       </c>
       <c r="D19" s="29" t="str">
         <f aca="false">IF(Models!D19="","",Models!D19)</f>
-        <v>China</v>
+        <v>France</v>
       </c>
       <c r="E19" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A19)</f>
@@ -4521,15 +4557,15 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="str">
         <f aca="false">IF(Models!A20="","",Models!A20)</f>
-        <v>minimax-m1</v>
+        <v>glm-4.5</v>
       </c>
       <c r="B20" s="29" t="str">
         <f aca="false">IF(Models!B20="","",Models!B20)</f>
-        <v>MiniMax-M1</v>
+        <v>GLM-4.5</v>
       </c>
       <c r="C20" s="29" t="str">
         <f aca="false">IF(Models!C20="","",Models!C20)</f>
-        <v>MiniMax</v>
+        <v>Zhipu AI / Z.ai</v>
       </c>
       <c r="D20" s="29" t="str">
         <f aca="false">IF(Models!D20="","",Models!D20)</f>
@@ -4587,15 +4623,15 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="29" t="str">
         <f aca="false">IF(Models!A21="","",Models!A21)</f>
-        <v>internlm3-8b</v>
+        <v>kimi-k2</v>
       </c>
       <c r="B21" s="29" t="str">
         <f aca="false">IF(Models!B21="","",Models!B21)</f>
-        <v>InternLM3 8B Instruct</v>
+        <v>Kimi K2 Instruct</v>
       </c>
       <c r="C21" s="29" t="str">
         <f aca="false">IF(Models!C21="","",Models!C21)</f>
-        <v>Shanghai AI Lab</v>
+        <v>Moonshot AI</v>
       </c>
       <c r="D21" s="29" t="str">
         <f aca="false">IF(Models!D21="","",Models!D21)</f>
@@ -4653,19 +4689,19 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="29" t="str">
         <f aca="false">IF(Models!A22="","",Models!A22)</f>
-        <v>aya-expanse-32b</v>
+        <v>minimax-m1</v>
       </c>
       <c r="B22" s="29" t="str">
         <f aca="false">IF(Models!B22="","",Models!B22)</f>
-        <v>Aya Expanse 32B</v>
+        <v>MiniMax-M1</v>
       </c>
       <c r="C22" s="29" t="str">
         <f aca="false">IF(Models!C22="","",Models!C22)</f>
-        <v>Cohere</v>
+        <v>MiniMax</v>
       </c>
       <c r="D22" s="29" t="str">
         <f aca="false">IF(Models!D22="","",Models!D22)</f>
-        <v>Canada</v>
+        <v>China</v>
       </c>
       <c r="E22" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A22)</f>
@@ -4719,19 +4755,19 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="29" t="str">
         <f aca="false">IF(Models!A23="","",Models!A23)</f>
-        <v>falcon3-10b</v>
+        <v>internlm3-8b</v>
       </c>
       <c r="B23" s="29" t="str">
         <f aca="false">IF(Models!B23="","",Models!B23)</f>
-        <v>Falcon 3 10B Instruct</v>
+        <v>InternLM3 8B Instruct</v>
       </c>
       <c r="C23" s="29" t="str">
         <f aca="false">IF(Models!C23="","",Models!C23)</f>
-        <v>TII</v>
+        <v>Shanghai AI Lab</v>
       </c>
       <c r="D23" s="29" t="str">
         <f aca="false">IF(Models!D23="","",Models!D23)</f>
-        <v>UAE</v>
+        <v>China</v>
       </c>
       <c r="E23" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A23)</f>
@@ -4785,19 +4821,19 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="29" t="str">
         <f aca="false">IF(Models!A24="","",Models!A24)</f>
-        <v>jamba-1.5-mini</v>
+        <v>aya-expanse-32b</v>
       </c>
       <c r="B24" s="29" t="str">
         <f aca="false">IF(Models!B24="","",Models!B24)</f>
-        <v>Jamba 1.5 Mini</v>
+        <v>Aya Expanse 32B</v>
       </c>
       <c r="C24" s="29" t="str">
         <f aca="false">IF(Models!C24="","",Models!C24)</f>
-        <v>AI21 Labs</v>
+        <v>Cohere</v>
       </c>
       <c r="D24" s="29" t="str">
         <f aca="false">IF(Models!D24="","",Models!D24)</f>
-        <v>Israel</v>
+        <v>Canada</v>
       </c>
       <c r="E24" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A24)</f>
@@ -4851,19 +4887,19 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="29" t="str">
         <f aca="false">IF(Models!A25="","",Models!A25)</f>
-        <v>exaone-4-32b</v>
+        <v>falcon3-10b</v>
       </c>
       <c r="B25" s="29" t="str">
         <f aca="false">IF(Models!B25="","",Models!B25)</f>
-        <v>EXAONE 4.0 32B</v>
+        <v>Falcon 3 10B Instruct</v>
       </c>
       <c r="C25" s="29" t="str">
         <f aca="false">IF(Models!C25="","",Models!C25)</f>
-        <v>LG AI Research</v>
+        <v>TII</v>
       </c>
       <c r="D25" s="29" t="str">
         <f aca="false">IF(Models!D25="","",Models!D25)</f>
-        <v>South Korea</v>
+        <v>UAE</v>
       </c>
       <c r="E25" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A25)</f>
@@ -4917,19 +4953,19 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="29" t="str">
         <f aca="false">IF(Models!A26="","",Models!A26)</f>
-        <v>sarvam-m</v>
+        <v>jamba-1.5-mini</v>
       </c>
       <c r="B26" s="29" t="str">
         <f aca="false">IF(Models!B26="","",Models!B26)</f>
-        <v>Sarvam-M</v>
+        <v>Jamba 1.5 Mini</v>
       </c>
       <c r="C26" s="29" t="str">
         <f aca="false">IF(Models!C26="","",Models!C26)</f>
-        <v>Sarvam AI</v>
+        <v>AI21 Labs</v>
       </c>
       <c r="D26" s="29" t="str">
         <f aca="false">IF(Models!D26="","",Models!D26)</f>
-        <v>India</v>
+        <v>Israel</v>
       </c>
       <c r="E26" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A26)</f>
@@ -4983,19 +5019,19 @@
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="29" t="str">
         <f aca="false">IF(Models!A27="","",Models!A27)</f>
-        <v>sea-lion-v3</v>
+        <v>exaone-4-32b</v>
       </c>
       <c r="B27" s="29" t="str">
         <f aca="false">IF(Models!B27="","",Models!B27)</f>
-        <v>SEA-LION v3 (Gemma-based)</v>
+        <v>EXAONE 4.0 32B</v>
       </c>
       <c r="C27" s="29" t="str">
         <f aca="false">IF(Models!C27="","",Models!C27)</f>
-        <v>AI Singapore</v>
+        <v>LG AI Research</v>
       </c>
       <c r="D27" s="29" t="str">
         <f aca="false">IF(Models!D27="","",Models!D27)</f>
-        <v>Singapore</v>
+        <v>South Korea</v>
       </c>
       <c r="E27" s="30" t="n">
         <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A27)</f>
@@ -5046,9 +5082,141 @@
         <v/>
       </c>
     </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="29" t="str">
+        <f aca="false">IF(Models!A28="","",Models!A28)</f>
+        <v>sarvam-m</v>
+      </c>
+      <c r="B28" s="29" t="str">
+        <f aca="false">IF(Models!B28="","",Models!B28)</f>
+        <v>Sarvam-M</v>
+      </c>
+      <c r="C28" s="29" t="str">
+        <f aca="false">IF(Models!C28="","",Models!C28)</f>
+        <v>Sarvam AI</v>
+      </c>
+      <c r="D28" s="29" t="str">
+        <f aca="false">IF(Models!D28="","",Models!D28)</f>
+        <v>India</v>
+      </c>
+      <c r="E28" s="30" t="n">
+        <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A28)</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="20" t="str">
+        <f aca="false">IF($E28=0,"",IFERROR(_xlfn.MAXIFS(Perf_Results!$AI$2:$AI$400,Perf_Results!$C$2:$C$400,$A28),""))</f>
+        <v/>
+      </c>
+      <c r="G28" s="20" t="str">
+        <f aca="false">IF($E28=0,"",IFERROR(_xlfn.MAXIFS(Perf_Results!$AS$2:$AS$400,Perf_Results!$C$2:$C$400,$A28),""))</f>
+        <v/>
+      </c>
+      <c r="H28" s="20" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Perf_Results!$Z$2:$Z$400,Perf_Results!$C$2:$C$400,$A28,Perf_Results!$O$2:$O$400,1),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="31" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Perf_Results!$AL$2:$AL$400,Perf_Results!$C$2:$C$400,$A28),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="32" t="str">
+        <f aca="false">IF($E28=0,"",IFERROR(_xlfn.MAXIFS(Perf_Results!$AU$2:$AU$400,Perf_Results!$C$2:$C$400,$A28),""))</f>
+        <v/>
+      </c>
+      <c r="K28" s="33" t="str">
+        <f aca="false">IF($E28=0,"",IFERROR(_xlfn.MINIFS(Perf_Results!$AW$2:$AW$400,Perf_Results!$C$2:$C$400,$A28),""))</f>
+        <v/>
+      </c>
+      <c r="L28" s="34" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Perf_Results!$AR$2:$AR$400,Perf_Results!$C$2:$C$400,$A28),"")</f>
+        <v/>
+      </c>
+      <c r="M28" s="30" t="n">
+        <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A28,Perf_Results!$AX$2:$AX$400,"PASS",Perf_Results!$AY$2:$AY$400,"PASS")</f>
+        <v>0</v>
+      </c>
+      <c r="N28" s="30" t="n">
+        <f aca="false">COUNTIFS(Quality_Results!$C$2:$C$300,$A28)</f>
+        <v>0</v>
+      </c>
+      <c r="O28" s="32" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Quality_Results!$Q$2:$Q$300,Quality_Results!$C$2:$C$300,$A28),"")</f>
+        <v/>
+      </c>
+      <c r="P28" s="31" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Quality_Results!$AF$2:$AF$300,Quality_Results!$C$2:$C$300,$A28),"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
-        <v>797</v>
+      <c r="A29" s="29" t="str">
+        <f aca="false">IF(Models!A29="","",Models!A29)</f>
+        <v>sea-lion-v3</v>
+      </c>
+      <c r="B29" s="29" t="str">
+        <f aca="false">IF(Models!B29="","",Models!B29)</f>
+        <v>SEA-LION v3 (Gemma-based)</v>
+      </c>
+      <c r="C29" s="29" t="str">
+        <f aca="false">IF(Models!C29="","",Models!C29)</f>
+        <v>AI Singapore</v>
+      </c>
+      <c r="D29" s="29" t="str">
+        <f aca="false">IF(Models!D29="","",Models!D29)</f>
+        <v>Singapore</v>
+      </c>
+      <c r="E29" s="30" t="n">
+        <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A29)</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="20" t="str">
+        <f aca="false">IF($E29=0,"",IFERROR(_xlfn.MAXIFS(Perf_Results!$AI$2:$AI$400,Perf_Results!$C$2:$C$400,$A29),""))</f>
+        <v/>
+      </c>
+      <c r="G29" s="20" t="str">
+        <f aca="false">IF($E29=0,"",IFERROR(_xlfn.MAXIFS(Perf_Results!$AS$2:$AS$400,Perf_Results!$C$2:$C$400,$A29),""))</f>
+        <v/>
+      </c>
+      <c r="H29" s="20" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Perf_Results!$Z$2:$Z$400,Perf_Results!$C$2:$C$400,$A29,Perf_Results!$O$2:$O$400,1),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="31" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Perf_Results!$AL$2:$AL$400,Perf_Results!$C$2:$C$400,$A29),"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="32" t="str">
+        <f aca="false">IF($E29=0,"",IFERROR(_xlfn.MAXIFS(Perf_Results!$AU$2:$AU$400,Perf_Results!$C$2:$C$400,$A29),""))</f>
+        <v/>
+      </c>
+      <c r="K29" s="33" t="str">
+        <f aca="false">IF($E29=0,"",IFERROR(_xlfn.MINIFS(Perf_Results!$AW$2:$AW$400,Perf_Results!$C$2:$C$400,$A29),""))</f>
+        <v/>
+      </c>
+      <c r="L29" s="34" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Perf_Results!$AR$2:$AR$400,Perf_Results!$C$2:$C$400,$A29),"")</f>
+        <v/>
+      </c>
+      <c r="M29" s="30" t="n">
+        <f aca="false">COUNTIFS(Perf_Results!$C$2:$C$400,$A29,Perf_Results!$AX$2:$AX$400,"PASS",Perf_Results!$AY$2:$AY$400,"PASS")</f>
+        <v>0</v>
+      </c>
+      <c r="N29" s="30" t="n">
+        <f aca="false">COUNTIFS(Quality_Results!$C$2:$C$300,$A29)</f>
+        <v>0</v>
+      </c>
+      <c r="O29" s="32" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Quality_Results!$Q$2:$Q$300,Quality_Results!$C$2:$C$300,$A29),"")</f>
+        <v/>
+      </c>
+      <c r="P29" s="31" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS(Quality_Results!$AF$2:$AF$300,Quality_Results!$C$2:$C$300,$A29),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>809</v>
       </c>
     </row>
   </sheetData>
@@ -8052,7 +8220,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -8624,7 +8792,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
         <v>600</v>
       </c>
@@ -8676,7 +8844,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
         <v>606</v>
       </c>
@@ -8684,7 +8852,7 @@
         <v>607</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>608</v>
+        <v>602</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>568</v>
@@ -8696,156 +8864,158 @@
         <v>498</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="I15" s="13" t="s">
         <v>561</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>4096</v>
+        <v>128000</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>555</v>
+        <v>608</v>
       </c>
       <c r="L15" s="13" t="s">
         <v>609</v>
       </c>
       <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
+      <c r="N15" s="13" t="s">
+        <v>610</v>
+      </c>
       <c r="O15" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P15" s="13" t="s">
-        <v>610</v>
+        <v>477</v>
       </c>
       <c r="Q15" s="13" t="s">
+        <v>580</v>
+      </c>
+      <c r="R15" s="14" t="s">
         <v>611</v>
       </c>
-      <c r="R15" s="14" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
         <v>612</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="B16" s="13" t="s">
         <v>613</v>
       </c>
-      <c r="B16" s="13" t="s">
-        <v>614</v>
-      </c>
       <c r="C16" s="13" t="s">
-        <v>615</v>
+        <v>602</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>616</v>
+        <v>568</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>539</v>
+        <v>569</v>
       </c>
       <c r="F16" s="13" t="s">
         <v>498</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="I16" s="13" t="s">
         <v>561</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>128000</v>
+        <v>4096</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>555</v>
+        <v>614</v>
       </c>
       <c r="L16" s="13" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="13" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="O16" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P16" s="13" t="s">
-        <v>477</v>
+        <v>617</v>
       </c>
       <c r="Q16" s="13" t="s">
-        <v>544</v>
-      </c>
-      <c r="R16" s="14"/>
+        <v>618</v>
+      </c>
+      <c r="R16" s="14" t="s">
+        <v>619</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>615</v>
+        <v>622</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>616</v>
+        <v>568</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>539</v>
+        <v>569</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>498</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>141</v>
+        <v>32</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>540</v>
+        <v>561</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>65536</v>
+        <v>4096</v>
       </c>
       <c r="K17" s="13" t="s">
         <v>555</v>
       </c>
       <c r="L17" s="13" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="M17" s="13"/>
-      <c r="N17" s="13" t="s">
-        <v>622</v>
-      </c>
+      <c r="N17" s="13"/>
       <c r="O17" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P17" s="13" t="s">
-        <v>543</v>
+        <v>617</v>
       </c>
       <c r="Q17" s="13" t="s">
-        <v>611</v>
+        <v>618</v>
       </c>
       <c r="R17" s="14" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>538</v>
+        <v>628</v>
       </c>
       <c r="E18" s="13" t="s">
         <v>539</v>
@@ -8854,50 +9024,50 @@
         <v>498</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>355</v>
+        <v>24</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>540</v>
+        <v>561</v>
       </c>
       <c r="J18" s="13" t="n">
         <v>128000</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="L18" s="13" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
+      <c r="N18" s="13" t="s">
+        <v>630</v>
+      </c>
       <c r="O18" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P18" s="13" t="s">
-        <v>543</v>
+        <v>477</v>
       </c>
       <c r="Q18" s="13" t="s">
-        <v>580</v>
-      </c>
-      <c r="R18" s="14" t="s">
-        <v>628</v>
-      </c>
+        <v>544</v>
+      </c>
+      <c r="R18" s="14"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>538</v>
+        <v>628</v>
       </c>
       <c r="E19" s="13" t="s">
         <v>539</v>
@@ -8906,33 +9076,35 @@
         <v>498</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>1000</v>
+        <v>141</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="I19" s="13" t="s">
         <v>540</v>
       </c>
       <c r="J19" s="13" t="n">
-        <v>128000</v>
+        <v>65536</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>632</v>
+        <v>555</v>
       </c>
       <c r="L19" s="13" t="s">
         <v>633</v>
       </c>
       <c r="M19" s="13"/>
-      <c r="N19" s="13"/>
+      <c r="N19" s="13" t="s">
+        <v>634</v>
+      </c>
       <c r="O19" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P19" s="13" t="s">
-        <v>634</v>
+        <v>543</v>
       </c>
       <c r="Q19" s="13" t="s">
-        <v>580</v>
+        <v>618</v>
       </c>
       <c r="R19" s="14" t="s">
         <v>635</v>
@@ -8958,19 +9130,19 @@
         <v>498</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>456</v>
+        <v>355</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="I20" s="13" t="s">
         <v>540</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>1000000</v>
+        <v>128000</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="L20" s="13" t="s">
         <v>639</v>
@@ -8981,10 +9153,10 @@
         <v>66</v>
       </c>
       <c r="P20" s="13" t="s">
-        <v>610</v>
+        <v>543</v>
       </c>
       <c r="Q20" s="13" t="s">
-        <v>611</v>
+        <v>580</v>
       </c>
       <c r="R20" s="14" t="s">
         <v>640</v>
@@ -9010,22 +9182,22 @@
         <v>498</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>8</v>
+        <v>1000</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>561</v>
+        <v>540</v>
       </c>
       <c r="J21" s="13" t="n">
-        <v>32768</v>
+        <v>128000</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>555</v>
+        <v>644</v>
       </c>
       <c r="L21" s="13" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
@@ -9033,25 +9205,27 @@
         <v>66</v>
       </c>
       <c r="P21" s="13" t="s">
-        <v>610</v>
+        <v>646</v>
       </c>
       <c r="Q21" s="13" t="s">
-        <v>611</v>
-      </c>
-      <c r="R21" s="14"/>
+        <v>580</v>
+      </c>
+      <c r="R21" s="14" t="s">
+        <v>647</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>648</v>
+        <v>538</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>539</v>
@@ -9060,35 +9234,33 @@
         <v>498</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>32</v>
+        <v>456</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="I22" s="13" t="s">
-        <v>561</v>
+        <v>540</v>
       </c>
       <c r="J22" s="13" t="n">
-        <v>128000</v>
+        <v>1000000</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>649</v>
+        <v>555</v>
       </c>
       <c r="L22" s="13" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="M22" s="13"/>
-      <c r="N22" s="13" t="s">
-        <v>651</v>
-      </c>
+      <c r="N22" s="13"/>
       <c r="O22" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P22" s="13" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="Q22" s="13" t="s">
-        <v>580</v>
+        <v>618</v>
       </c>
       <c r="R22" s="14" t="s">
         <v>652</v>
@@ -9105,7 +9277,7 @@
         <v>655</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>656</v>
+        <v>538</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>539</v>
@@ -9114,10 +9286,10 @@
         <v>498</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H23" s="13" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I23" s="13" t="s">
         <v>561</v>
@@ -9126,38 +9298,36 @@
         <v>32768</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>657</v>
+        <v>555</v>
       </c>
       <c r="L23" s="13" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="M23" s="13"/>
-      <c r="N23" s="13" t="s">
-        <v>659</v>
-      </c>
+      <c r="N23" s="13"/>
       <c r="O23" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P23" s="13" t="s">
-        <v>660</v>
+        <v>617</v>
       </c>
       <c r="Q23" s="13" t="s">
-        <v>611</v>
+        <v>618</v>
       </c>
       <c r="R23" s="14"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="E24" s="13" t="s">
         <v>539</v>
@@ -9166,50 +9336,52 @@
         <v>498</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="H24" s="13" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>665</v>
+        <v>561</v>
       </c>
       <c r="J24" s="13" t="n">
-        <v>256000</v>
+        <v>128000</v>
       </c>
       <c r="K24" s="13" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
       <c r="L24" s="13" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="M24" s="13"/>
-      <c r="N24" s="13"/>
+      <c r="N24" s="13" t="s">
+        <v>663</v>
+      </c>
       <c r="O24" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P24" s="13" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="Q24" s="13" t="s">
-        <v>611</v>
+        <v>580</v>
       </c>
       <c r="R24" s="14" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="E25" s="13" t="s">
         <v>539</v>
@@ -9218,50 +9390,50 @@
         <v>498</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="H25" s="13" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="I25" s="13" t="s">
         <v>561</v>
       </c>
       <c r="J25" s="13" t="n">
-        <v>128000</v>
+        <v>32768</v>
       </c>
       <c r="K25" s="13" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="L25" s="13" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="M25" s="13"/>
-      <c r="N25" s="13"/>
+      <c r="N25" s="13" t="s">
+        <v>671</v>
+      </c>
       <c r="O25" s="13" t="s">
         <v>66</v>
       </c>
       <c r="P25" s="13" t="s">
-        <v>610</v>
+        <v>672</v>
       </c>
       <c r="Q25" s="13" t="s">
-        <v>611</v>
-      </c>
-      <c r="R25" s="14" t="s">
+        <v>618</v>
+      </c>
+      <c r="R25" s="14"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
+        <v>673</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>674</v>
+      </c>
+      <c r="C26" s="13" t="s">
         <v>675</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
+      <c r="D26" s="13" t="s">
         <v>676</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>677</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>678</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>679</v>
       </c>
       <c r="E26" s="13" t="s">
         <v>539</v>
@@ -9270,22 +9442,22 @@
         <v>498</v>
       </c>
       <c r="G26" s="13" t="n">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="H26" s="13" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="I26" s="13" t="s">
-        <v>561</v>
+        <v>677</v>
       </c>
       <c r="J26" s="13" t="n">
-        <v>32768</v>
+        <v>256000</v>
       </c>
       <c r="K26" s="13" t="s">
-        <v>555</v>
+        <v>678</v>
       </c>
       <c r="L26" s="13" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
@@ -9293,27 +9465,27 @@
         <v>66</v>
       </c>
       <c r="P26" s="13" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="Q26" s="13" t="s">
-        <v>580</v>
+        <v>618</v>
       </c>
       <c r="R26" s="14" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
+        <v>681</v>
+      </c>
+      <c r="B27" s="13" t="s">
         <v>682</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="C27" s="13" t="s">
         <v>683</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="D27" s="13" t="s">
         <v>684</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>685</v>
       </c>
       <c r="E27" s="13" t="s">
         <v>539</v>
@@ -9322,19 +9494,19 @@
         <v>498</v>
       </c>
       <c r="G27" s="13" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H27" s="13" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="I27" s="13" t="s">
         <v>561</v>
       </c>
       <c r="J27" s="13" t="n">
-        <v>8192</v>
+        <v>128000</v>
       </c>
       <c r="K27" s="13" t="s">
-        <v>591</v>
+        <v>685</v>
       </c>
       <c r="L27" s="13" t="s">
         <v>686</v>
@@ -9345,22 +9517,126 @@
         <v>66</v>
       </c>
       <c r="P27" s="13" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="Q27" s="13" t="s">
-        <v>611</v>
+        <v>618</v>
       </c>
       <c r="R27" s="14" t="s">
         <v>687</v>
       </c>
     </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
+        <v>688</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>689</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>690</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>691</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>539</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>498</v>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="H28" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="I28" s="13" t="s">
+        <v>561</v>
+      </c>
+      <c r="J28" s="13" t="n">
+        <v>32768</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>555</v>
+      </c>
+      <c r="L28" s="13" t="s">
+        <v>692</v>
+      </c>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
+      <c r="O28" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="P28" s="13" t="s">
+        <v>617</v>
+      </c>
+      <c r="Q28" s="13" t="s">
+        <v>580</v>
+      </c>
+      <c r="R28" s="14" t="s">
+        <v>693</v>
+      </c>
+    </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
-        <v>688</v>
+      <c r="A29" s="13" t="s">
+        <v>694</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>695</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>696</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>697</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>539</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>498</v>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="H29" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="I29" s="13" t="s">
+        <v>561</v>
+      </c>
+      <c r="J29" s="13" t="n">
+        <v>8192</v>
+      </c>
+      <c r="K29" s="13" t="s">
+        <v>591</v>
+      </c>
+      <c r="L29" s="13" t="s">
+        <v>698</v>
+      </c>
+      <c r="M29" s="13"/>
+      <c r="N29" s="13"/>
+      <c r="O29" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="P29" s="13" t="s">
+        <v>617</v>
+      </c>
+      <c r="Q29" s="13" t="s">
+        <v>618</v>
+      </c>
+      <c r="R29" s="14" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="s">
+        <v>700</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:R27"/>
+  <autoFilter ref="A4:R29"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -9394,17 +9670,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>689</v>
+        <v>701</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>690</v>
+        <v>702</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>691</v>
+        <v>703</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>65</v>
@@ -9413,28 +9689,28 @@
         <v>531</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>692</v>
+        <v>704</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>693</v>
+        <v>705</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>694</v>
+        <v>706</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>695</v>
+        <v>707</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>696</v>
+        <v>708</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>697</v>
+        <v>709</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>698</v>
+        <v>710</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>699</v>
+        <v>711</v>
       </c>
     </row>
   </sheetData>
@@ -9466,17 +9742,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>700</v>
+        <v>712</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>369</v>
@@ -9485,7 +9761,7 @@
         <v>58</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9499,7 +9775,7 @@
         <v>233</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>704</v>
+        <v>716</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9513,12 +9789,12 @@
         <v>242</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>705</v>
+        <v>717</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>706</v>
+        <v>718</v>
       </c>
       <c r="B7" s="17" t="n">
         <v>8</v>
@@ -9527,7 +9803,7 @@
         <v>106</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>707</v>
+        <v>719</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9541,7 +9817,7 @@
         <v>193</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9555,7 +9831,7 @@
         <v>251</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>709</v>
+        <v>721</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9569,7 +9845,7 @@
         <v>256</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>710</v>
+        <v>722</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9588,7 +9864,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>711</v>
+        <v>723</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>0.15</v>
@@ -9597,12 +9873,12 @@
         <v>193</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>712</v>
+        <v>724</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>713</v>
+        <v>725</v>
       </c>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -9610,92 +9886,92 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>714</v>
+        <v>726</v>
       </c>
       <c r="B15" s="19" t="n">
         <f aca="false">B5/B6</f>
         <v>87500</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>715</v>
+        <v>727</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>716</v>
+        <v>728</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>717</v>
+        <v>729</v>
       </c>
       <c r="B16" s="19" t="n">
         <f aca="false">B5*B12</f>
         <v>52500</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>715</v>
+        <v>727</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>718</v>
+        <v>730</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>719</v>
+        <v>731</v>
       </c>
       <c r="B17" s="20" t="n">
         <f aca="false">B9*B10*8760*B8</f>
         <v>87564.96</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>720</v>
+        <v>732</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>721</v>
+        <v>733</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>722</v>
+        <v>734</v>
       </c>
       <c r="B18" s="19" t="n">
         <f aca="false">B17*B11</f>
         <v>7880.8464</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>715</v>
+        <v>727</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>723</v>
+        <v>735</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>724</v>
+        <v>736</v>
       </c>
       <c r="B19" s="19" t="n">
         <f aca="false">B15+B16+B18</f>
         <v>147880.8464</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>715</v>
+        <v>727</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>725</v>
+        <v>737</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>726</v>
+        <v>738</v>
       </c>
       <c r="B20" s="20" t="n">
         <f aca="false">B7*8760*B8</f>
         <v>49056</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>727</v>
+        <v>739</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9710,7 +9986,7 @@
         <v>233</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>729</v>
+        <v>741</v>
       </c>
     </row>
   </sheetData>
@@ -9741,10 +10017,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>730</v>
+        <v>742</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>691</v>
+        <v>703</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>65</v>
@@ -9759,7 +10035,7 @@
         <v>101</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>731</v>
+        <v>743</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>105</v>
@@ -9768,7 +10044,7 @@
         <v>109</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>732</v>
+        <v>744</v>
       </c>
       <c r="K1" s="7" t="s">
         <v>378</v>
@@ -9801,43 +10077,43 @@
         <v>148</v>
       </c>
       <c r="U1" s="7" t="s">
-        <v>733</v>
+        <v>745</v>
       </c>
       <c r="V1" s="7" t="s">
-        <v>734</v>
+        <v>746</v>
       </c>
       <c r="W1" s="7" t="s">
-        <v>735</v>
+        <v>747</v>
       </c>
       <c r="X1" s="7" t="s">
-        <v>736</v>
+        <v>748</v>
       </c>
       <c r="Y1" s="7" t="s">
-        <v>737</v>
+        <v>749</v>
       </c>
       <c r="Z1" s="7" t="s">
-        <v>738</v>
+        <v>750</v>
       </c>
       <c r="AA1" s="7" t="s">
-        <v>739</v>
+        <v>751</v>
       </c>
       <c r="AB1" s="7" t="s">
-        <v>740</v>
+        <v>752</v>
       </c>
       <c r="AC1" s="7" t="s">
-        <v>741</v>
+        <v>753</v>
       </c>
       <c r="AD1" s="7" t="s">
         <v>162</v>
       </c>
       <c r="AE1" s="7" t="s">
-        <v>742</v>
+        <v>754</v>
       </c>
       <c r="AF1" s="7" t="s">
-        <v>743</v>
+        <v>755</v>
       </c>
       <c r="AG1" s="7" t="s">
-        <v>744</v>
+        <v>756</v>
       </c>
       <c r="AH1" s="7" t="s">
         <v>169</v>
@@ -9858,10 +10134,10 @@
         <v>192</v>
       </c>
       <c r="AN1" s="7" t="s">
-        <v>745</v>
+        <v>757</v>
       </c>
       <c r="AO1" s="7" t="s">
-        <v>746</v>
+        <v>758</v>
       </c>
       <c r="AP1" s="7" t="s">
         <v>123</v>
@@ -9899,25 +10175,25 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>747</v>
+        <v>759</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>748</v>
+        <v>760</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>749</v>
+        <v>761</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>750</v>
+        <v>762</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>751</v>
+        <v>763</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>752</v>
+        <v>764</v>
       </c>
       <c r="G2" s="22" t="s">
-        <v>753</v>
+        <v>765</v>
       </c>
       <c r="H2" s="22" t="n">
         <v>2</v>
@@ -9926,7 +10202,7 @@
         <v>1</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>754</v>
+        <v>766</v>
       </c>
       <c r="K2" s="22" t="n">
         <v>2</v>
@@ -9935,10 +10211,10 @@
         <v>32768</v>
       </c>
       <c r="M2" s="22" t="s">
-        <v>755</v>
+        <v>767</v>
       </c>
       <c r="N2" s="22" t="s">
-        <v>756</v>
+        <v>768</v>
       </c>
       <c r="O2" s="22" t="n">
         <v>32</v>
@@ -10058,7 +10334,7 @@
         <v>PASS</v>
       </c>
       <c r="AZ2" s="22" t="s">
-        <v>757</v>
+        <v>769</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23638,10 +23914,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>730</v>
+        <v>742</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>691</v>
+        <v>703</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>65</v>
@@ -23653,49 +23929,49 @@
         <v>101</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>758</v>
+        <v>770</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>759</v>
+        <v>771</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>760</v>
+        <v>772</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>302</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>761</v>
+        <v>773</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>762</v>
+        <v>774</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>763</v>
+        <v>775</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>490</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>764</v>
+        <v>776</v>
       </c>
       <c r="O1" s="7" t="s">
         <v>330</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>765</v>
+        <v>777</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>272</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>766</v>
+        <v>778</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>767</v>
+        <v>779</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>768</v>
+        <v>780</v>
       </c>
       <c r="U1" s="7" t="s">
         <v>282</v>
@@ -23716,19 +23992,19 @@
         <v>321</v>
       </c>
       <c r="AA1" s="7" t="s">
-        <v>769</v>
+        <v>781</v>
       </c>
       <c r="AB1" s="7" t="s">
         <v>317</v>
       </c>
       <c r="AC1" s="7" t="s">
-        <v>770</v>
+        <v>782</v>
       </c>
       <c r="AD1" s="7" t="s">
-        <v>771</v>
+        <v>783</v>
       </c>
       <c r="AE1" s="7" t="s">
-        <v>772</v>
+        <v>784</v>
       </c>
       <c r="AF1" s="7" t="s">
         <v>314</v>
@@ -23739,31 +24015,31 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>773</v>
+        <v>785</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>774</v>
+        <v>786</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>749</v>
+        <v>761</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>752</v>
+        <v>764</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>775</v>
+        <v>787</v>
       </c>
       <c r="G2" s="22" t="s">
-        <v>776</v>
+        <v>788</v>
       </c>
       <c r="H2" s="22" t="s">
-        <v>777</v>
+        <v>789</v>
       </c>
       <c r="I2" s="22" t="s">
-        <v>778</v>
+        <v>790</v>
       </c>
       <c r="J2" s="22" t="n">
         <v>1000</v>
@@ -23784,7 +24060,7 @@
         <v>42</v>
       </c>
       <c r="P2" s="22" t="s">
-        <v>779</v>
+        <v>791</v>
       </c>
       <c r="Q2" s="22" t="n">
         <v>0.712</v>
@@ -23818,10 +24094,10 @@
         <v>4.9</v>
       </c>
       <c r="AB2" s="22" t="s">
-        <v>780</v>
+        <v>792</v>
       </c>
       <c r="AC2" s="22" t="s">
-        <v>781</v>
+        <v>793</v>
       </c>
       <c r="AD2" s="25" t="n">
         <f aca="false">IFERROR(1.96*R2/SQRT(J2*K2),"")</f>
@@ -23836,7 +24112,7 @@
         <v>0</v>
       </c>
       <c r="AG2" s="22" t="s">
-        <v>782</v>
+        <v>794</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>